<commit_message>
Ažurirao statistike prema XLSX
</commit_message>
<xml_diff>
--- a/public/data/KK_Posusje_statistika_25-26.xlsx
+++ b/public/data/KK_Posusje_statistika_25-26.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FOI\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59CB7E62-FE95-47A2-B0EA-1187C3BCB078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24BFD5BD-9771-41F0-8653-617F4ADDDEF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Players" sheetId="1" r:id="rId1"/>
     <sheet name="Team Stats" sheetId="2" r:id="rId2"/>
-    <sheet name="Games" sheetId="3" r:id="rId3"/>
+    <sheet name="Games" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="118">
   <si>
     <t>Player</t>
   </si>
@@ -158,6 +158,27 @@
     <t>TO_per_game</t>
   </si>
   <si>
+    <t>DR_per_game</t>
+  </si>
+  <si>
+    <t>OR_per_game</t>
+  </si>
+  <si>
+    <t>STL_per_game</t>
+  </si>
+  <si>
+    <t>BLK_per_game</t>
+  </si>
+  <si>
+    <t>PF_per_game</t>
+  </si>
+  <si>
+    <t>3P_per_game</t>
+  </si>
+  <si>
+    <t>3PA_per_game</t>
+  </si>
+  <si>
     <t>Ante Kovač</t>
   </si>
   <si>
@@ -215,9 +236,39 @@
     <t>Points</t>
   </si>
   <si>
+    <t>FG</t>
+  </si>
+  <si>
+    <t>386/851</t>
+  </si>
+  <si>
+    <t>2P</t>
+  </si>
+  <si>
+    <t>242/436</t>
+  </si>
+  <si>
+    <t>3P</t>
+  </si>
+  <si>
+    <t>124/383</t>
+  </si>
+  <si>
+    <t>FT</t>
+  </si>
+  <si>
+    <t>114/197</t>
+  </si>
+  <si>
     <t>Rebounds</t>
   </si>
   <si>
+    <t>DR</t>
+  </si>
+  <si>
+    <t>OR</t>
+  </si>
+  <si>
     <t>Assists</t>
   </si>
   <si>
@@ -233,24 +284,6 @@
     <t>Fouls</t>
   </si>
   <si>
-    <t>FG</t>
-  </si>
-  <si>
-    <t>386/851</t>
-  </si>
-  <si>
-    <t>3P</t>
-  </si>
-  <si>
-    <t>124/383</t>
-  </si>
-  <si>
-    <t>FT</t>
-  </si>
-  <si>
-    <t>114/197</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -272,12 +305,24 @@
     <t>Result</t>
   </si>
   <si>
+    <t>08.03.2026</t>
+  </si>
+  <si>
+    <t>Liga KSHB</t>
+  </si>
+  <si>
+    <t>KK Posušje</t>
+  </si>
+  <si>
+    <t>HKK Grude</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
     <t>02.11.2025</t>
   </si>
   <si>
-    <t>Liga KSHB</t>
-  </si>
-  <si>
     <t>HKK Posušje</t>
   </si>
   <si>
@@ -299,9 +344,6 @@
     <t>HKK Široki II</t>
   </si>
   <si>
-    <t>W</t>
-  </si>
-  <si>
     <t>23.11.2025</t>
   </si>
   <si>
@@ -311,9 +353,6 @@
     <t>30.11.2025</t>
   </si>
   <si>
-    <t>HKK Grude</t>
-  </si>
-  <si>
     <t>07.12.2025</t>
   </si>
   <si>
@@ -342,12 +381,6 @@
   </si>
   <si>
     <t>01.03.2026</t>
-  </si>
-  <si>
-    <t>KK Posušje</t>
-  </si>
-  <si>
-    <t>08.03.2026</t>
   </si>
 </sst>
 </file>
@@ -412,14 +445,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalno" xfId="0" builtinId="0"/>
@@ -722,13 +756,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AU20"/>
+  <dimension ref="A1:AX16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="1" max="1" width="14.109375" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -858,14 +893,31 @@
       <c r="AQ1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="1"/>
-      <c r="AS1" s="1"/>
-      <c r="AT1" s="1"/>
-      <c r="AU1" s="1"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B2" s="1">
         <v>13</v>
@@ -910,7 +962,7 @@
         <v>175</v>
       </c>
       <c r="P2" s="1">
-        <v>0.44</v>
+        <v>0.43430000000000002</v>
       </c>
       <c r="Q2" s="1">
         <v>37</v>
@@ -919,7 +971,7 @@
         <v>66</v>
       </c>
       <c r="S2" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.56059999999999999</v>
       </c>
       <c r="T2" s="1">
         <v>38</v>
@@ -928,7 +980,7 @@
         <v>107</v>
       </c>
       <c r="V2" s="1">
-        <v>0.36</v>
+        <v>0.35510000000000003</v>
       </c>
       <c r="W2" s="1">
         <v>12</v>
@@ -973,13 +1025,13 @@
         <v>8.42</v>
       </c>
       <c r="AK2" s="1">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="AL2" s="1">
-        <v>0.54</v>
+        <v>0.54290000000000005</v>
       </c>
       <c r="AM2" s="1">
-        <v>0.55000000000000004</v>
+        <v>0.54949999999999999</v>
       </c>
       <c r="AN2" s="1">
         <v>15.54</v>
@@ -993,14 +1045,31 @@
       <c r="AQ2" s="1">
         <v>1.77</v>
       </c>
-      <c r="AR2" s="1"/>
-      <c r="AS2" s="1"/>
-      <c r="AT2" s="1"/>
-      <c r="AU2" s="1"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR2" s="1">
+        <v>4.2300000000000004</v>
+      </c>
+      <c r="AS2" s="1">
+        <v>1.38</v>
+      </c>
+      <c r="AT2" s="1">
+        <v>1.69</v>
+      </c>
+      <c r="AU2" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="AV2" s="1">
+        <v>3.31</v>
+      </c>
+      <c r="AW2" s="1">
+        <v>2.92</v>
+      </c>
+      <c r="AX2" s="1">
+        <v>8.23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="B3" s="1">
         <v>12</v>
@@ -1045,7 +1114,7 @@
         <v>147</v>
       </c>
       <c r="P3" s="1">
-        <v>0.42</v>
+        <v>0.42859999999999998</v>
       </c>
       <c r="Q3" s="1">
         <v>33</v>
@@ -1054,7 +1123,7 @@
         <v>63</v>
       </c>
       <c r="S3" s="1">
-        <v>0.52</v>
+        <v>0.52380000000000004</v>
       </c>
       <c r="T3" s="1">
         <v>23</v>
@@ -1063,7 +1132,7 @@
         <v>75</v>
       </c>
       <c r="V3" s="1">
-        <v>0.33</v>
+        <v>0.30669999999999997</v>
       </c>
       <c r="W3" s="1">
         <v>35</v>
@@ -1072,7 +1141,7 @@
         <v>51</v>
       </c>
       <c r="Y3" s="1">
-        <v>0.67</v>
+        <v>0.68630000000000002</v>
       </c>
       <c r="Z3" s="1">
         <v>14.82</v>
@@ -1108,13 +1177,13 @@
         <v>6</v>
       </c>
       <c r="AK3" s="1">
-        <v>173</v>
+        <v>197</v>
       </c>
       <c r="AL3" s="1">
-        <v>0.51</v>
+        <v>0.50680000000000003</v>
       </c>
       <c r="AM3" s="1">
-        <v>0.54</v>
+        <v>0.54300000000000004</v>
       </c>
       <c r="AN3" s="1">
         <v>15.33</v>
@@ -1128,14 +1197,31 @@
       <c r="AQ3" s="1">
         <v>1.92</v>
       </c>
-      <c r="AR3" s="1"/>
-      <c r="AS3" s="1"/>
-      <c r="AT3" s="1"/>
-      <c r="AU3" s="1"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR3" s="1">
+        <v>4.42</v>
+      </c>
+      <c r="AS3" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AT3" s="1">
+        <v>1.17</v>
+      </c>
+      <c r="AU3" s="1">
+        <v>0.08</v>
+      </c>
+      <c r="AV3" s="1">
+        <v>2.42</v>
+      </c>
+      <c r="AW3" s="1">
+        <v>1.92</v>
+      </c>
+      <c r="AX3" s="1">
+        <v>6.25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="B4" s="1">
         <v>13</v>
@@ -1180,7 +1266,7 @@
         <v>142</v>
       </c>
       <c r="P4" s="1">
-        <v>0.39</v>
+        <v>0.40139999999999998</v>
       </c>
       <c r="Q4" s="1">
         <v>10</v>
@@ -1198,7 +1284,7 @@
         <v>117</v>
       </c>
       <c r="V4" s="1">
-        <v>0.38</v>
+        <v>0.4017</v>
       </c>
       <c r="W4" s="1">
         <v>8</v>
@@ -1207,7 +1293,7 @@
         <v>14</v>
       </c>
       <c r="Y4" s="1">
-        <v>0.5</v>
+        <v>0.57140000000000002</v>
       </c>
       <c r="Z4" s="1">
         <v>12.17</v>
@@ -1243,13 +1329,13 @@
         <v>8.67</v>
       </c>
       <c r="AK4" s="1">
-        <v>177</v>
+        <v>202</v>
       </c>
       <c r="AL4" s="1">
-        <v>0.54</v>
+        <v>0.56689999999999996</v>
       </c>
       <c r="AM4" s="1">
-        <v>0.54</v>
+        <v>0.57030000000000003</v>
       </c>
       <c r="AN4" s="1">
         <v>13</v>
@@ -1263,14 +1349,31 @@
       <c r="AQ4" s="1">
         <v>1.85</v>
       </c>
-      <c r="AR4" s="1"/>
-      <c r="AS4" s="1"/>
-      <c r="AT4" s="1"/>
-      <c r="AU4" s="1"/>
-    </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR4" s="1">
+        <v>5.69</v>
+      </c>
+      <c r="AS4" s="1">
+        <v>1.23</v>
+      </c>
+      <c r="AT4" s="1">
+        <v>1.46</v>
+      </c>
+      <c r="AU4" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="AV4" s="1">
+        <v>2.46</v>
+      </c>
+      <c r="AW4" s="1">
+        <v>3.62</v>
+      </c>
+      <c r="AX4" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="B5" s="1">
         <v>13</v>
@@ -1315,7 +1418,7 @@
         <v>107</v>
       </c>
       <c r="P5" s="1">
-        <v>0.46</v>
+        <v>0.47660000000000002</v>
       </c>
       <c r="Q5" s="1">
         <v>41</v>
@@ -1324,7 +1427,7 @@
         <v>66</v>
       </c>
       <c r="S5" s="1">
-        <v>0.62</v>
+        <v>0.62119999999999997</v>
       </c>
       <c r="T5" s="1">
         <v>4</v>
@@ -1333,7 +1436,7 @@
         <v>32</v>
       </c>
       <c r="V5" s="1">
-        <v>0.13</v>
+        <v>0.125</v>
       </c>
       <c r="W5" s="1">
         <v>13</v>
@@ -1378,13 +1481,13 @@
         <v>2.58</v>
       </c>
       <c r="AK5" s="1">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="AL5" s="1">
-        <v>0.48</v>
+        <v>0.49530000000000002</v>
       </c>
       <c r="AM5" s="1">
-        <v>0.49</v>
+        <v>0.50419999999999998</v>
       </c>
       <c r="AN5" s="1">
         <v>9.15</v>
@@ -1398,14 +1501,31 @@
       <c r="AQ5" s="1">
         <v>1.62</v>
       </c>
-      <c r="AR5" s="1"/>
-      <c r="AS5" s="1"/>
-      <c r="AT5" s="1"/>
-      <c r="AU5" s="1"/>
-    </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR5" s="1">
+        <v>5.15</v>
+      </c>
+      <c r="AS5" s="1">
+        <v>1.31</v>
+      </c>
+      <c r="AT5" s="1">
+        <v>0.69</v>
+      </c>
+      <c r="AU5" s="1">
+        <v>1.23</v>
+      </c>
+      <c r="AV5" s="1">
+        <v>2.54</v>
+      </c>
+      <c r="AW5" s="1">
+        <v>0.31</v>
+      </c>
+      <c r="AX5" s="1">
+        <v>2.46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B6" s="1">
         <v>12</v>
@@ -1450,7 +1570,7 @@
         <v>82</v>
       </c>
       <c r="P6" s="1">
-        <v>0.51</v>
+        <v>0.52439999999999998</v>
       </c>
       <c r="Q6" s="1">
         <v>36</v>
@@ -1468,7 +1588,7 @@
         <v>3</v>
       </c>
       <c r="V6" s="1">
-        <v>0.67</v>
+        <v>0.66669999999999996</v>
       </c>
       <c r="W6" s="1">
         <v>11</v>
@@ -1477,7 +1597,7 @@
         <v>22</v>
       </c>
       <c r="Y6" s="1">
-        <v>0.55000000000000004</v>
+        <v>0.5</v>
       </c>
       <c r="Z6" s="1">
         <v>8.09</v>
@@ -1513,13 +1633,13 @@
         <v>0.27</v>
       </c>
       <c r="AK6" s="1">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="AL6" s="1">
-        <v>0.52</v>
+        <v>0.53659999999999997</v>
       </c>
       <c r="AM6" s="1">
-        <v>0.53</v>
+        <v>0.53990000000000005</v>
       </c>
       <c r="AN6" s="1">
         <v>8.25</v>
@@ -1533,14 +1653,31 @@
       <c r="AQ6" s="1">
         <v>1.5</v>
       </c>
-      <c r="AR6" s="1"/>
-      <c r="AS6" s="1"/>
-      <c r="AT6" s="1"/>
-      <c r="AU6" s="1"/>
-    </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR6" s="1">
+        <v>2.25</v>
+      </c>
+      <c r="AS6" s="1">
+        <v>1.67</v>
+      </c>
+      <c r="AT6" s="1">
+        <v>0.17</v>
+      </c>
+      <c r="AU6" s="1">
+        <v>0</v>
+      </c>
+      <c r="AV6" s="1">
+        <v>2.67</v>
+      </c>
+      <c r="AW6" s="1">
+        <v>0.17</v>
+      </c>
+      <c r="AX6" s="1">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="B7" s="1">
         <v>13</v>
@@ -1585,7 +1722,7 @@
         <v>54</v>
       </c>
       <c r="P7" s="1">
-        <v>0.45</v>
+        <v>0.46300000000000002</v>
       </c>
       <c r="Q7" s="1">
         <v>23</v>
@@ -1594,7 +1731,7 @@
         <v>41</v>
       </c>
       <c r="S7" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.56100000000000005</v>
       </c>
       <c r="T7" s="1">
         <v>1</v>
@@ -1612,7 +1749,7 @@
         <v>19</v>
       </c>
       <c r="Y7" s="1">
-        <v>0.53</v>
+        <v>0.52629999999999999</v>
       </c>
       <c r="Z7" s="1">
         <v>4.67</v>
@@ -1648,13 +1785,13 @@
         <v>0.83</v>
       </c>
       <c r="AK7" s="1">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="AL7" s="1">
-        <v>0.46</v>
+        <v>0.47220000000000001</v>
       </c>
       <c r="AM7" s="1">
-        <v>0.46</v>
+        <v>0.46500000000000002</v>
       </c>
       <c r="AN7" s="1">
         <v>4.46</v>
@@ -1668,14 +1805,31 @@
       <c r="AQ7" s="1">
         <v>0.77</v>
       </c>
-      <c r="AR7" s="1"/>
-      <c r="AS7" s="1"/>
-      <c r="AT7" s="1"/>
-      <c r="AU7" s="1"/>
-    </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR7" s="1">
+        <v>2.85</v>
+      </c>
+      <c r="AS7" s="1">
+        <v>1</v>
+      </c>
+      <c r="AT7" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="AU7" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="AV7" s="1">
+        <v>2.08</v>
+      </c>
+      <c r="AW7" s="1">
+        <v>0.08</v>
+      </c>
+      <c r="AX7" s="1">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B8" s="1">
         <v>12</v>
@@ -1720,7 +1874,7 @@
         <v>35</v>
       </c>
       <c r="P8" s="1">
-        <v>0.78</v>
+        <v>0.71430000000000005</v>
       </c>
       <c r="Q8" s="1">
         <v>25</v>
@@ -1729,7 +1883,7 @@
         <v>29</v>
       </c>
       <c r="S8" s="1">
-        <v>0.86</v>
+        <v>0.86209999999999998</v>
       </c>
       <c r="T8" s="1">
         <v>0</v>
@@ -1783,13 +1937,13 @@
         <v>0.27</v>
       </c>
       <c r="AK8" s="1">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="AL8" s="1">
-        <v>0.78</v>
+        <v>0.71430000000000005</v>
       </c>
       <c r="AM8" s="1">
-        <v>0.73</v>
+        <v>0.67310000000000003</v>
       </c>
       <c r="AN8" s="1">
         <v>4.67</v>
@@ -1803,14 +1957,31 @@
       <c r="AQ8" s="1">
         <v>0.83</v>
       </c>
-      <c r="AR8" s="1"/>
-      <c r="AS8" s="1"/>
-      <c r="AT8" s="1"/>
-      <c r="AU8" s="1"/>
-    </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR8" s="1">
+        <v>2.42</v>
+      </c>
+      <c r="AS8" s="1">
+        <v>1.75</v>
+      </c>
+      <c r="AT8" s="1">
+        <v>0.92</v>
+      </c>
+      <c r="AU8" s="1">
+        <v>0.08</v>
+      </c>
+      <c r="AV8" s="1">
+        <v>3.25</v>
+      </c>
+      <c r="AW8" s="1">
+        <v>0</v>
+      </c>
+      <c r="AX8" s="1">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="B9" s="1">
         <v>9</v>
@@ -1855,7 +2026,7 @@
         <v>47</v>
       </c>
       <c r="P9" s="1">
-        <v>0.36</v>
+        <v>0.31909999999999999</v>
       </c>
       <c r="Q9" s="1">
         <v>11</v>
@@ -1864,7 +2035,7 @@
         <v>27</v>
       </c>
       <c r="S9" s="1">
-        <v>0.41</v>
+        <v>0.40739999999999998</v>
       </c>
       <c r="T9" s="1">
         <v>4</v>
@@ -1873,7 +2044,7 @@
         <v>17</v>
       </c>
       <c r="V9" s="1">
-        <v>0.27</v>
+        <v>0.23530000000000001</v>
       </c>
       <c r="W9" s="1">
         <v>14</v>
@@ -1882,7 +2053,7 @@
         <v>19</v>
       </c>
       <c r="Y9" s="1">
-        <v>0.74</v>
+        <v>0.73680000000000001</v>
       </c>
       <c r="Z9" s="1">
         <v>5.62</v>
@@ -1918,13 +2089,13 @@
         <v>1.38</v>
       </c>
       <c r="AK9" s="1">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AL9" s="1">
-        <v>0.4</v>
+        <v>0.36170000000000002</v>
       </c>
       <c r="AM9" s="1">
-        <v>0.48</v>
+        <v>0.4335</v>
       </c>
       <c r="AN9" s="1">
         <v>5.33</v>
@@ -1938,14 +2109,31 @@
       <c r="AQ9" s="1">
         <v>1.33</v>
       </c>
-      <c r="AR9" s="1"/>
-      <c r="AS9" s="1"/>
-      <c r="AT9" s="1"/>
-      <c r="AU9" s="1"/>
-    </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR9" s="1">
+        <v>1.33</v>
+      </c>
+      <c r="AS9" s="1">
+        <v>0.78</v>
+      </c>
+      <c r="AT9" s="1">
+        <v>0.89</v>
+      </c>
+      <c r="AU9" s="1">
+        <v>0</v>
+      </c>
+      <c r="AV9" s="1">
+        <v>1.33</v>
+      </c>
+      <c r="AW9" s="1">
+        <v>0.44</v>
+      </c>
+      <c r="AX9" s="1">
+        <v>1.89</v>
+      </c>
+    </row>
+    <row r="10" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B10" s="1">
         <v>8</v>
@@ -1990,7 +2178,7 @@
         <v>23</v>
       </c>
       <c r="P10" s="1">
-        <v>0.48</v>
+        <v>0.4783</v>
       </c>
       <c r="Q10" s="1">
         <v>10</v>
@@ -1999,7 +2187,7 @@
         <v>18</v>
       </c>
       <c r="S10" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.55559999999999998</v>
       </c>
       <c r="T10" s="1">
         <v>1</v>
@@ -2008,7 +2196,7 @@
         <v>6</v>
       </c>
       <c r="V10" s="1">
-        <v>0.17</v>
+        <v>0.16669999999999999</v>
       </c>
       <c r="W10" s="1">
         <v>3</v>
@@ -2059,7 +2247,7 @@
         <v>0.5</v>
       </c>
       <c r="AM10" s="1">
-        <v>0.51</v>
+        <v>0.50700000000000001</v>
       </c>
       <c r="AN10" s="1">
         <v>3.25</v>
@@ -2073,14 +2261,31 @@
       <c r="AQ10" s="1">
         <v>0.75</v>
       </c>
-      <c r="AR10" s="1"/>
-      <c r="AS10" s="1"/>
-      <c r="AT10" s="1"/>
-      <c r="AU10" s="1"/>
-    </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR10" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="AS10" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AT10" s="1">
+        <v>0</v>
+      </c>
+      <c r="AU10" s="1">
+        <v>0</v>
+      </c>
+      <c r="AV10" s="1">
+        <v>1.38</v>
+      </c>
+      <c r="AW10" s="1">
+        <v>0.12</v>
+      </c>
+      <c r="AX10" s="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B11" s="1">
         <v>8</v>
@@ -2125,7 +2330,7 @@
         <v>18</v>
       </c>
       <c r="P11" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.55559999999999998</v>
       </c>
       <c r="Q11" s="1">
         <v>9</v>
@@ -2134,7 +2339,7 @@
         <v>16</v>
       </c>
       <c r="S11" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.5625</v>
       </c>
       <c r="T11" s="1">
         <v>1</v>
@@ -2143,7 +2348,7 @@
         <v>3</v>
       </c>
       <c r="V11" s="1">
-        <v>0.33</v>
+        <v>0.33329999999999999</v>
       </c>
       <c r="W11" s="1">
         <v>1</v>
@@ -2191,10 +2396,10 @@
         <v>18</v>
       </c>
       <c r="AL11" s="1">
-        <v>0.57999999999999996</v>
+        <v>0.58330000000000004</v>
       </c>
       <c r="AM11" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.55669999999999997</v>
       </c>
       <c r="AN11" s="1">
         <v>2.75</v>
@@ -2208,14 +2413,31 @@
       <c r="AQ11" s="1">
         <v>0.88</v>
       </c>
-      <c r="AR11" s="1"/>
-      <c r="AS11" s="1"/>
-      <c r="AT11" s="1"/>
-      <c r="AU11" s="1"/>
-    </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR11" s="1">
+        <v>0.62</v>
+      </c>
+      <c r="AS11" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="AT11" s="1">
+        <v>0.62</v>
+      </c>
+      <c r="AU11" s="1">
+        <v>0</v>
+      </c>
+      <c r="AV11" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="AW11" s="1">
+        <v>0.12</v>
+      </c>
+      <c r="AX11" s="1">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="B12" s="1">
         <v>3</v>
@@ -2260,7 +2482,7 @@
         <v>8</v>
       </c>
       <c r="P12" s="1">
-        <v>0.38</v>
+        <v>0.375</v>
       </c>
       <c r="Q12" s="1">
         <v>0</v>
@@ -2278,7 +2500,7 @@
         <v>8</v>
       </c>
       <c r="V12" s="1">
-        <v>0.38</v>
+        <v>0.375</v>
       </c>
       <c r="W12" s="1">
         <v>0</v>
@@ -2326,10 +2548,10 @@
         <v>2</v>
       </c>
       <c r="AL12" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.5625</v>
       </c>
       <c r="AM12" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.5625</v>
       </c>
       <c r="AN12" s="1">
         <v>3</v>
@@ -2343,14 +2565,31 @@
       <c r="AQ12" s="1">
         <v>1</v>
       </c>
-      <c r="AR12" s="1"/>
-      <c r="AS12" s="1"/>
-      <c r="AT12" s="1"/>
-      <c r="AU12" s="1"/>
-    </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR12" s="1">
+        <v>0</v>
+      </c>
+      <c r="AS12" s="1">
+        <v>0.33</v>
+      </c>
+      <c r="AT12" s="1">
+        <v>0</v>
+      </c>
+      <c r="AU12" s="1">
+        <v>0</v>
+      </c>
+      <c r="AV12" s="1">
+        <v>0.33</v>
+      </c>
+      <c r="AW12" s="1">
+        <v>1</v>
+      </c>
+      <c r="AX12" s="1">
+        <v>2.67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B13" s="1">
         <v>1</v>
@@ -2395,7 +2634,7 @@
         <v>7</v>
       </c>
       <c r="P13" s="1">
-        <v>0.56999999999999995</v>
+        <v>0.57140000000000002</v>
       </c>
       <c r="Q13" s="1">
         <v>4</v>
@@ -2404,7 +2643,7 @@
         <v>7</v>
       </c>
       <c r="S13" s="1">
-        <v>0.56999999999999995</v>
+        <v>0.57140000000000002</v>
       </c>
       <c r="T13" s="1">
         <v>0</v>
@@ -2461,10 +2700,10 @@
         <v>6</v>
       </c>
       <c r="AL13" s="1">
-        <v>0.56999999999999995</v>
+        <v>0.57140000000000002</v>
       </c>
       <c r="AM13" s="1">
-        <v>0.56999999999999995</v>
+        <v>0.57110000000000005</v>
       </c>
       <c r="AN13" s="1">
         <v>9</v>
@@ -2478,14 +2717,31 @@
       <c r="AQ13" s="1">
         <v>1</v>
       </c>
-      <c r="AR13" s="1"/>
-      <c r="AS13" s="1"/>
-      <c r="AT13" s="1"/>
-      <c r="AU13" s="1"/>
-    </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR13" s="1">
+        <v>0</v>
+      </c>
+      <c r="AS13" s="1">
+        <v>1</v>
+      </c>
+      <c r="AT13" s="1">
+        <v>0</v>
+      </c>
+      <c r="AU13" s="1">
+        <v>0</v>
+      </c>
+      <c r="AV13" s="1">
+        <v>0</v>
+      </c>
+      <c r="AW13" s="1">
+        <v>0</v>
+      </c>
+      <c r="AX13" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="B14" s="1">
         <v>2</v>
@@ -2613,14 +2869,31 @@
       <c r="AQ14" s="1">
         <v>0.5</v>
       </c>
-      <c r="AR14" s="1"/>
-      <c r="AS14" s="1"/>
-      <c r="AT14" s="1"/>
-      <c r="AU14" s="1"/>
-    </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR14" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="AS14" s="1">
+        <v>0</v>
+      </c>
+      <c r="AT14" s="1">
+        <v>0</v>
+      </c>
+      <c r="AU14" s="1">
+        <v>0</v>
+      </c>
+      <c r="AV14" s="1">
+        <v>0</v>
+      </c>
+      <c r="AW14" s="1">
+        <v>0</v>
+      </c>
+      <c r="AX14" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B15" s="1">
         <v>1</v>
@@ -2748,14 +3021,31 @@
       <c r="AQ15" s="1">
         <v>3</v>
       </c>
-      <c r="AR15" s="1"/>
-      <c r="AS15" s="1"/>
-      <c r="AT15" s="1"/>
-      <c r="AU15" s="1"/>
-    </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="AR15" s="1">
+        <v>0</v>
+      </c>
+      <c r="AS15" s="1">
+        <v>0</v>
+      </c>
+      <c r="AT15" s="1">
+        <v>0</v>
+      </c>
+      <c r="AU15" s="1">
+        <v>0</v>
+      </c>
+      <c r="AV15" s="1">
+        <v>3</v>
+      </c>
+      <c r="AW15" s="1">
+        <v>0</v>
+      </c>
+      <c r="AX15" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B16" s="1">
         <v>1</v>
@@ -2883,206 +3173,27 @@
       <c r="AQ16" s="1">
         <v>0</v>
       </c>
-      <c r="AR16" s="1"/>
-      <c r="AS16" s="1"/>
-      <c r="AT16" s="1"/>
-      <c r="AU16" s="1"/>
-    </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
-      <c r="Q17" s="1"/>
-      <c r="R17" s="1"/>
-      <c r="S17" s="1"/>
-      <c r="T17" s="1"/>
-      <c r="U17" s="1"/>
-      <c r="V17" s="1"/>
-      <c r="W17" s="1"/>
-      <c r="X17" s="1"/>
-      <c r="Y17" s="1"/>
-      <c r="Z17" s="1"/>
-      <c r="AA17" s="1"/>
-      <c r="AB17" s="1"/>
-      <c r="AC17" s="1"/>
-      <c r="AD17" s="1"/>
-      <c r="AE17" s="1"/>
-      <c r="AF17" s="1"/>
-      <c r="AG17" s="1"/>
-      <c r="AH17" s="1"/>
-      <c r="AI17" s="1"/>
-      <c r="AJ17" s="1"/>
-      <c r="AK17" s="1"/>
-      <c r="AL17" s="1"/>
-      <c r="AM17" s="1"/>
-      <c r="AN17" s="1"/>
-      <c r="AO17" s="1"/>
-      <c r="AP17" s="1"/>
-      <c r="AQ17" s="1"/>
-      <c r="AR17" s="1"/>
-      <c r="AS17" s="1"/>
-      <c r="AT17" s="1"/>
-      <c r="AU17" s="1"/>
-    </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
-      <c r="Q18" s="1"/>
-      <c r="R18" s="1"/>
-      <c r="S18" s="1"/>
-      <c r="T18" s="1"/>
-      <c r="U18" s="1"/>
-      <c r="V18" s="1"/>
-      <c r="W18" s="1"/>
-      <c r="X18" s="1"/>
-      <c r="Y18" s="1"/>
-      <c r="Z18" s="1"/>
-      <c r="AA18" s="1"/>
-      <c r="AB18" s="1"/>
-      <c r="AC18" s="1"/>
-      <c r="AD18" s="1"/>
-      <c r="AE18" s="1"/>
-      <c r="AF18" s="1"/>
-      <c r="AG18" s="1"/>
-      <c r="AH18" s="1"/>
-      <c r="AI18" s="1"/>
-      <c r="AJ18" s="1"/>
-      <c r="AK18" s="1"/>
-      <c r="AL18" s="1"/>
-      <c r="AM18" s="1"/>
-      <c r="AN18" s="1"/>
-      <c r="AO18" s="1"/>
-      <c r="AP18" s="1"/>
-      <c r="AQ18" s="1"/>
-      <c r="AR18" s="1"/>
-      <c r="AS18" s="1"/>
-      <c r="AT18" s="1"/>
-      <c r="AU18" s="1"/>
-    </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
-      <c r="Q19" s="1"/>
-      <c r="R19" s="1"/>
-      <c r="S19" s="1"/>
-      <c r="T19" s="1"/>
-      <c r="U19" s="1"/>
-      <c r="V19" s="1"/>
-      <c r="W19" s="1"/>
-      <c r="X19" s="1"/>
-      <c r="Y19" s="1"/>
-      <c r="Z19" s="1"/>
-      <c r="AA19" s="1"/>
-      <c r="AB19" s="1"/>
-      <c r="AC19" s="1"/>
-      <c r="AD19" s="1"/>
-      <c r="AE19" s="1"/>
-      <c r="AF19" s="1"/>
-      <c r="AG19" s="1"/>
-      <c r="AH19" s="1"/>
-      <c r="AI19" s="1"/>
-      <c r="AJ19" s="1"/>
-      <c r="AK19" s="1"/>
-      <c r="AL19" s="1"/>
-      <c r="AM19" s="1"/>
-      <c r="AN19" s="1"/>
-      <c r="AO19" s="1"/>
-      <c r="AP19" s="1"/>
-      <c r="AQ19" s="1"/>
-      <c r="AR19" s="1"/>
-      <c r="AS19" s="1"/>
-      <c r="AT19" s="1"/>
-      <c r="AU19" s="1"/>
-    </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
-      <c r="P20" s="1"/>
-      <c r="Q20" s="1"/>
-      <c r="R20" s="1"/>
-      <c r="S20" s="1"/>
-      <c r="T20" s="1"/>
-      <c r="U20" s="1"/>
-      <c r="V20" s="1"/>
-      <c r="W20" s="1"/>
-      <c r="X20" s="1"/>
-      <c r="Y20" s="1"/>
-      <c r="Z20" s="1"/>
-      <c r="AA20" s="1"/>
-      <c r="AB20" s="1"/>
-      <c r="AC20" s="1"/>
-      <c r="AD20" s="1"/>
-      <c r="AE20" s="1"/>
-      <c r="AF20" s="1"/>
-      <c r="AG20" s="1"/>
-      <c r="AH20" s="1"/>
-      <c r="AI20" s="1"/>
-      <c r="AJ20" s="1"/>
-      <c r="AK20" s="1"/>
-      <c r="AL20" s="1"/>
-      <c r="AM20" s="1"/>
-      <c r="AN20" s="1"/>
-      <c r="AO20" s="1"/>
-      <c r="AP20" s="1"/>
-      <c r="AQ20" s="1"/>
-      <c r="AR20" s="1"/>
-      <c r="AS20" s="1"/>
-      <c r="AT20" s="1"/>
-      <c r="AU20" s="1"/>
+      <c r="AR16" s="1">
+        <v>0</v>
+      </c>
+      <c r="AS16" s="1">
+        <v>0</v>
+      </c>
+      <c r="AT16" s="1">
+        <v>0</v>
+      </c>
+      <c r="AU16" s="1">
+        <v>0</v>
+      </c>
+      <c r="AV16" s="1">
+        <v>0</v>
+      </c>
+      <c r="AW16" s="1">
+        <v>0</v>
+      </c>
+      <c r="AX16" s="1">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3091,252 +3202,184 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B2" s="1">
         <v>13</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B3" s="1">
         <v>1007</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B4" s="1">
         <v>77.459999999999994</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" s="1">
+        <v>69</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="1">
+        <v>45.36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="1">
+        <v>55.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="1">
+        <v>32.380000000000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="1">
+        <v>57.87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" s="1">
         <v>491</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="1">
-        <v>37.770000000000003</v>
-      </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B7" s="1">
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="1">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="1">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" s="1">
         <v>210</v>
       </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="1">
-        <v>16.149999999999999</v>
-      </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B9" s="1">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" s="1">
         <v>162</v>
       </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" s="1">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B19" s="1">
         <v>30</v>
       </c>
-      <c r="B10" s="1">
-        <v>12.46</v>
-      </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B11" s="1">
-        <v>95</v>
-      </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B12" s="1">
-        <v>30</v>
-      </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B13" s="1">
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="1">
         <v>265</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15" s="1">
-        <v>45.36</v>
-      </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="1">
-        <v>32.380000000000003</v>
-      </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="1">
-        <v>57.87</v>
-      </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="1">
+        <v>52.64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="1">
+        <v>53.7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3344,7 +3387,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3359,372 +3402,375 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D2" s="3">
+        <v>81</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F2" s="3">
+        <v>85</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" s="3">
+        <v>92</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" s="3">
+        <v>78</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D4" s="3">
+        <v>79</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F4" s="3">
+        <v>72</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="3">
+        <v>90</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="F5" s="3">
         <v>77</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G1" s="2" t="s">
+      <c r="G5" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="3">
+        <v>60</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F6" s="3">
+        <v>56</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D7" s="3">
+        <v>33</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" s="3">
+        <v>107</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D8" s="3">
+        <v>85</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F8" s="3">
+        <v>81</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D9" s="3">
+        <v>54</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F9" s="3">
+        <v>69</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D10" s="3">
+        <v>60</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F10" s="3">
+        <v>55</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D11" s="3">
+        <v>90</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="F11" s="3">
+        <v>84</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D12" s="3">
+        <v>70</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F12" s="3">
+        <v>62</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D13" s="3">
+        <v>60</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F13" s="3">
+        <v>94</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D14" s="3">
         <v>80</v>
       </c>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D2" s="1">
-        <v>81</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="F2" s="1">
-        <v>85</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="1">
-        <v>92</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F3" s="1">
-        <v>78</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D4" s="1">
-        <v>79</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="F4" s="1">
-        <v>72</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D5" s="1">
-        <v>90</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F5" s="1">
-        <v>77</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="D6" s="1">
-        <v>60</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F6" s="1">
-        <v>56</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="E14" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C7" s="1" t="s">
+      <c r="F14" s="3">
+        <v>67</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="1">
-        <v>33</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F7" s="1">
-        <v>107</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="D8" s="1">
-        <v>85</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F8" s="1">
-        <v>81</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D9" s="1">
-        <v>54</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="F9" s="1">
-        <v>69</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D10" s="1">
-        <v>60</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F10" s="1">
-        <v>55</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D11" s="1">
-        <v>90</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="F11" s="1">
-        <v>84</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D12" s="1">
-        <v>70</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F12" s="1">
-        <v>62</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D13" s="1">
-        <v>60</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="F13" s="1">
-        <v>94</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D14" s="1">
-        <v>80</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="F14" s="1">
-        <v>67</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H14" s="1"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>